<commit_message>
Approve Sponsored Brands/video test; add competitor landscape to doc and workbooks
Corrections doc: new sections on the competitive landscape (what it
confirms and changes in the push) and the approved Sponsored Brands /
video test; summary, new-campaign decisions and next steps updated.
Campaign workbook: SB & video test and Competitive landscape tabs; the
audit's SB/SBV/SD builds decided. Engine reference: SB & video test tab,
approvals reflected in gaps, rules, overview and validation plan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LY7A1KPDoE1cQtWdmceR2R
</commit_message>
<xml_diff>
--- a/docs/B6_Campaign_Decisions_20260929.xlsx
+++ b/docs/B6_Campaign_Decisions_20260929.xlsx
@@ -13,10 +13,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign decisions" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit rows" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New campaigns" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By hand" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Negatives" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SB &amp; video test" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitive landscape" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By hand" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Negatives" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Campaign decisions'!$A$4:$AR$366</definedName>
@@ -557,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -596,14 +598,14 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>It applies the same rules as the corrections document. Where this sheet and the audit disagree, this sheet applies. Tabs: In-depth analysis · Push plan · Campaign decisions (every campaign) · Audit rows (all 188, each with a verdict) · New campaigns (the 17 builds) · By hand (colour, objective, budgets, restarts) · Negatives · Timeline · Checks.</t>
+          <t>It applies the same rules as the corrections document. Where this sheet and the audit disagree, this sheet applies. Tabs: In-depth analysis · Push plan · Campaign decisions (every campaign) · Audit rows (all 188, each with a verdict) · New campaigns (the 17 builds) · SB &amp; video test (approved) · Competitive landscape · By hand (colour, objective, budgets, restarts) · Negatives · Timeline · Checks.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Sources: the audit export; Command Center (30 and 90 days to 29 Sep, placements; deal days 26–28 Sep); Sellerboard margins per colour (27 Aug–25 Sep, profit before ads) and stock; our daily rank crawl (29 Sep).</t>
+          <t>Sources: the audit export; Command Center (30 and 90 days to 29 Sep, placements; deal days 26–28 Sep); Sellerboard margins per colour (27 Aug–25 Sep, profit before ads) and stock; our daily rank crawl (29 Sep); ASINsight competitor exports (13 rivals, 28–29 Sep) and Data Dive niches (16–29 Sep).</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1119,24 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Spend limit and the margin rule after the deal; the 17 new campaigns; restarts; the two structural folds; the brand negatives on the Decolure broad.</t>
+          <t>Spend limit and the margin rule after the deal; the other new campaigns; restarts; the two structural folds; the brand negatives on the Decolure broad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>Decided 29 Sep</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Sponsored Brands / video test</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Approved: 6 hand-built campaigns from 1 Oct at break-even bids, $85 a day for 14 days as a separate budget line (SB &amp; video test tab).</t>
         </is>
       </c>
     </row>
@@ -1133,6 +1152,817 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Negative keywords — one campaign per search term</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Every ranking term is bought by one exact campaign; broad, auto and phrase campaigns exclude it</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Seq</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Negatives now</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>After</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Terms added (negative exact)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Our verdict</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n">
+        <v>1738</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo sheets king size-[Bamboo|King]-(HSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>1 term(s)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>1966</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo sheets king size-[Bamboo|King]-(HSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>36 term(s)</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>10 term(s)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="n">
+        <v>1967</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo cooling sheets-[Bamboo|Cooling]-(MSV)-Broad-(DISC)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>13 term(s)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>8 term(s)</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n">
+        <v>1968</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo sheets queen size-[Bamboo|Queen]-(HSV)-Broad-(DISC)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>33 term(s)</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>7 term(s)</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n">
+        <v>1969</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo sheets full-[Bamboo|Full]-(MSV)-Broad-(DISC)-DO-BAMBOO-FULL-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>20 term(s)</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>10 term(s)</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>1970</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>SP-Luxury Womens Gifts-(NOSV)-Broad-(Discovery)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>3 term(s)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>3 term(s)</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
+        <v>1971</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo sheets california king-[Bamboo|California King]-(LSV)-Broad-(DISC)-DO-BAMBOO-CALIFKING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>7 term(s)</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>4 term(s)</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>1972</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo sheets-[Bamboo]-(VHSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>0 term(s)</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>43 term(s)</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n">
+        <v>1974</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>SP-Auto-(AUTO)-Auto-(Discovery)-DO-BAMBOO-KING-TAUPE-6PCS</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>127 term(s)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>17 term(s)</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>1976</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>SP-Queen Sheets-(VHSV)-Broad-(Discovery)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>0 term(s)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>15 term(s)</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n">
+        <v>1977</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>SP-Auto-(AUTO)-Auto-(Discovery)-DO-BAMBOO-QUEEN-OLIVE-6PCS-3</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>18 term(s)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>50 term(s)</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>2142</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>SP-Decolure-(VLSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>10 term(s)</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>2 term(s)</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>brand negatives wait until the three brand exact campaigns are defensive and serving</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>2143</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo sheets california king-[Bamboo|California King]-(LSV)-Broad-(DISC)-DO-BAMBOO-CALIFKING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>7 term(s)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1 term(s)</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>2144</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>SP-Auto-(AUTO)-Auto-(Discovery)-DO-BAMBOO-KING-TAUPE-6PCS</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>127 term(s)</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>2 term(s)</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n">
+        <v>2145</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo sheets full-[Bamboo|Full]-(MSV)-Broad-(DISC)-DO-BAMBOO-FULL-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>20 term(s)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>2 term(s)</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>2146</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo sheets-[Bamboo]-(VHSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>0 term(s)</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1 term(s)</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
+        <v>2147</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>SP-bamboo cooling sheets-[Bamboo|Cooling]-(MSV)-Broad-(DISC)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>13 term(s)</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1 term(s)</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr"/>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>2148</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>SP-Auto-(AUTO)-Auto-(Discovery)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>136 term(s)</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1 term(s)</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>one campaign per term: excludes terms an exact campaign owns</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Also exclude “bamboo sheets” (negative exact) from every broad discovery campaign that still buys it; the “bamboo sheets” exact campaign owns it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A24:J24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="150" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timeline — deal exit and the next events</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>29–30 Sep (deal)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Load the 13 push terms (base + boost in one write, budgets by hand); cuts to break-even on non-push ranking campaigns; base cuts on conversions/discovery over break-even on 30 and 90 days; restart “bamboo sheets full”. Colour switches to White by hand on push campaigns first. Hold every new campaign, fold and the brand negatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>1 Oct — post-deal audit</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Confirm regular price; re-price on the full-price margin ($18.81). Re-evaluate the spend limit and the margin rule. Bring deal budgets down to each campaign’s required clicks at its new price. Decide the other builds, the restarts and the folds. Push carries on without a gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>1 Oct — SB &amp; video test starts</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Build SB-1, SBV-2–4, SB-5 and SD-6 by hand at break-even bids; $85 a day for 14 days, separate budget line. Daily: +30% bid step while a banner isn’t showing, never above twice break-even.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>1–7 Oct — watch, don’t judge</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Deal-click sales keep arriving until ~7 Oct. Daily: spend vs limit, ad orders vs 14/day, top-of-search share on push campaigns, head-term ranks, Full White and Queen White stock. A head term falling &gt;10 places → find the cause before touching price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>5 Oct</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>First weekly push tune.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>8–14 Oct — first clean read</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Re-run break-even on seven normal days. Mix check: where product pages still take &gt;20%, cut base again. Tune push on 12 Oct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>14 Oct — SB &amp; video test read</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Per campaign on ≥15 clicks: keep at or below break-even; hold at break-even bid between break-even and twice; stop above. Check the same-term SP campaign didn’t lose orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>15 Oct — Lightning Deal</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>One day. Don’t judge on it; keep push prices; check budgets won’t run out by mid-afternoon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>19 Oct</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Weekly tune. Goal: top 10 on at least half the push terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>22–28 Oct — Best Deal</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Size the push for the deal a week ahead (price, clicks, budget, stock). The day-28 rank read skips deal days. Queen White arrival (1,002) lands 30 Oct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>From early Nov</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Push into Prime / Black Friday–Cyber Monday: each event sized, funded and stock-checked at least three weeks ahead.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -67048,7 +67878,7 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Hold. Decide 1 Oct after the listing check: one Sponsored Brands format per term, not both.</t>
+          <t>BUILD 1 Oct as SBV-3 in the SB &amp; video test: video, King White, break-even bid $3.19, $15/day.</t>
         </is>
       </c>
     </row>
@@ -67088,7 +67918,7 @@
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Hold. Decide 1 Oct after the listing check; pick this headline format or the video, not both.</t>
+          <t>Don’t build: one format per term — the video (1886) is chosen.</t>
         </is>
       </c>
     </row>
@@ -67128,7 +67958,7 @@
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Hold. Push term; decide 1 Oct whether it gets a single Sponsored Brands format once its top-of-search share moves.</t>
+          <t>BUILD 1 Oct as SBV-4 in the SB &amp; video test: video, Queen White, break-even bid $3.17, $12/day.</t>
         </is>
       </c>
     </row>
@@ -67168,7 +67998,7 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Hold. Rank 36 → 9, not in the push; decide 1 Oct.</t>
+          <t>Don’t build: one format per cooling term — the video on “bamboo cooling sheets” (1902) is chosen.</t>
         </is>
       </c>
     </row>
@@ -67208,7 +68038,7 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Build 1 Oct as the single Sponsored Brands support for a push term (pick video or headline).</t>
+          <t>BUILD 1 Oct as SBV-2 in the SB &amp; video test: video, Queen White, break-even bid $3.17, $15/day.</t>
         </is>
       </c>
     </row>
@@ -67248,7 +68078,7 @@
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Build 1 Oct only if the video (1918) is not chosen.</t>
+          <t>Don’t build: one format per term — the video (1918) is chosen.</t>
         </is>
       </c>
     </row>
@@ -67288,7 +68118,7 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Build 1 Oct as the single Sponsored Brands support for a push term (pick video or headline).</t>
+          <t>Don’t build: we already out-rank every tracked rival on “bamboo sheets full” and Full White stock is 68 units.</t>
         </is>
       </c>
     </row>
@@ -67328,7 +68158,7 @@
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Build 1 Oct only if the video (1934) is not chosen.</t>
+          <t>Don’t build: we already out-rank every tracked rival on “bamboo sheets full” and Full White stock is 68 units.</t>
         </is>
       </c>
     </row>
@@ -67368,7 +68198,7 @@
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Build 1 Oct: defends our own listing pages at low cost; budget inside the 1 Oct limit.</t>
+          <t>BUILD 1 Oct as SD-6 in the SB &amp; video test: own product pages, break-even bid $3.19, $10/day.</t>
         </is>
       </c>
     </row>
@@ -67408,7 +68238,7 @@
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>Build 1 Oct as a test with its own budget line inside the 1 Oct limit; judged on its own ACoS.</t>
+          <t>Build 1 Oct as a test with its own budget line, limited to the OFFENSIVE competitor ASINs (Competitive landscape tab); judged on its own ACoS.</t>
         </is>
       </c>
     </row>
@@ -67877,6 +68707,2132 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sponsored Brands and video test — approved 29 September, starts 1 October</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Built by hand; $85 a day for 14 days as a separate budget line; break-even bids</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Keyword(s) — exact</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Advertised colour</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Creative lands on</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Audit build</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Rivals with a headline</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Rivals with video</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Start bid $</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Ceiling $</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Budget $/day</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>SB-1</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Sponsored Brands — product collection (headline)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>bamboo sheets</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>King White</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>King White, Queen White, King Light Blue → product collection</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>new (no audit build)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>B6’s biggest term (1.16M market traffic). 5 rivals run a headline banner and 5 run video above our top-of-search slot. Headline first: the collection shows the 6-piece range in one banner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>SBV-2</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Sponsored Brands video</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>bamboo sheets queen size</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Queen White</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Queen White product page</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>build 1918 (video) — build 1926 (headline) not built</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>7 rivals run video on it, 5 a headline; the video slot is the one the field uses most.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>SBV-3</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Sponsored Brands video</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>bamboo sheets king size</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>King White</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>King White product page</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>build 1886 (video) — build 1894 (headline) not built</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Waiting SP term (ceiling below cost): the video banner tests the term at break-even without lifting the SP ceiling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>SBV-4</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Sponsored Brands video</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>bamboo cooling sheets</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Queen White</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Queen White product page</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>build 1902 (video) — build 1910 (headline on “bamboo cooling sheets king size”) not built</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>8 rivals run video on it — the most of any push term — and cooling is our most uncovered wording.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>SB-5</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Sponsored Brands — store spotlight (headline)</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>decolure bamboo sheets, decolure bamboo sheets king size, decolure</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>King White</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Decolure Store</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>new (no audit build)</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Brand defence: 10 rivals advertise on “decolure bamboo sheets”, 4 with a headline and 7 with video; the banner above our own name should be ours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>SD-6</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Sponsored Display — own product pages</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>B6 product pages (20 child ASINs)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>King White</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Own B6 pages</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>build 1950 (own-page defence)</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
+      <c r="I10" s="7" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Keeps rivals’ ads off our own product pages (rivals show on 1,000–3,500 keywords through product-page ads).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="8" t="n"/>
+      <c r="K11" s="7" t="n">
+        <v>85</v>
+      </c>
+      <c r="L11" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Start (1 Oct)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Bid = break-even of the advertised colour: margin × the size’s top-of-search conversion (King White $15.97 × 20.0% = $3.19; Queen White $19.51 × 16.2% = $3.17). Exact match only. Bidding strategy left as it is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Daily while the banner isn’t showing</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Raise the bid ≤30% a day, never above twice break-even (King $6.38, Queen $6.34).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>At 15 clicks</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Replace the size rate with the campaign’s own conversion (blended 15–50 clicks, own from 50), as for Sponsored Products; break-even and the ceiling move with it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>20 clicks, 0 orders on a keyword</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Pause the keyword.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>ACoS over twice break-even on ≥30 clicks</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Back to break-even bid; pause if it stays there 7 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Read on 14 Oct (before the 15 Oct Lightning Deal)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>ACoS at or below break-even ACoS (the 1 Oct audit re-sets it on the full-price margin): keep, and let the budget grow ≤30% a step. Between break-even and twice break-even: keep at the break-even bid. Above twice break-even: stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Halo check (same dates)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>The Sponsored Products campaign on the same term: orders and top-of-search conversion not below the 7 days before the test; organic rank not worse. If SP orders fall by more than the SB orders add, the banner is taking our own clicks: stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Impressions, click-through, cost per click, orders, ACoS, new-to-brand share, and for SB-5 the rivals’ share of “decolure bamboo sheets” in the next ASINsight export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>• Built by hand in Campaign Manager (the engine’s write path is Sponsored Products only), registered as a cross-format pair with the SP campaign on the same term.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>• Separate budget line: $85 a day for 14 days (about $1,190), counted in B6’s total spend limit from 1 October but not in the SP push budgets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>• Headline creative: “6-piece bamboo sheet set — 2 extra pillowcases” (the value-per-piece position against 4-piece sets at $80–135); brand logo; no price claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>• Video: 15–30 seconds, the set in use (softness, cooling), the 6 pieces laid out, ending on the product. If no video is ready on 1 October, SBV-2 to SBV-4 run as headline until it is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>• No new negatives; exact match keeps each banner on its one term.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A25:J25"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="80" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Competitive landscape — what it changes in these decisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ASINsight: 13 measured rivals, all 2,225 addressable keywords (28–29 Sep); Data Dive: 3 niches (16–29 Sep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Push, waiting and at-target terms in their competitive field</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Our organic (ASINsight)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Tracked rivals ranked (top 5)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Rivals with a brand banner</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Our paid share</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Market paid share</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>bamboo sheets</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #3, Pure Bamboo #9, KRIMANO #17, Bambaw #19, BC Bella Coterie #20</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — stretch target</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Only Aspirational rivals hold rank 9 or better (Bedsure (cooling) #3, Pure Bamboo #9); target is a stretch — judge progress on the Beatable rivals we pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>bamboo sheets queen size</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #4, Pure Bamboo #12, KRIMANO #13, Bambaw #14, BC Bella Coterie #20</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — stretch target</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Only Aspirational rivals hold rank 5 or better (Bedsure (cooling) #4); target is a stretch — judge progress on the Beatable rivals we pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>bamboo sheets king size</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>WAIT</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #4, KRIMANO #6, Pure Bamboo #11, SONORO KATE (deep) #26, BC Bella Coterie #28</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>0.368</v>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — reachable</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>KRIMANO #6 (Beatable) already holds a rank at or above target #10: the target is reachable for a listing like ours. Rivals to pass first: Pure Bamboo #11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>bamboo sheets king</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>WAIT</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Pure Bamboo #4, KRIMANO #9, SONORO KATE (deep) #20, BC Bella Coterie #22, Bambaw #24</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>0.438</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — reachable</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>KRIMANO #9 (Beatable) already holds a rank at or above target #9: the target is reachable for a listing like ours. Rivals to pass first: SONORO KATE (deep) #20, BC Bella Coterie #22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>bamboo cooling sheets</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #2, Pure Bamboo #8, Bambaw #11, KRIMANO #19, BC Bella Coterie #22</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>0.384</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — stretch target</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Only Aspirational rivals hold rank 5 or better (Bedsure (cooling) #2); target is a stretch — judge progress on the Beatable rivals we pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>bamboo bed sheets</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>WAIT</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #2, Pure Bamboo #5, Bambaw #8, KRIMANO #9, BC Bella Coterie #20</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>0.354</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — stretch target</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Only Aspirational rivals hold rank 6 or better (Bedsure (cooling) #2, Pure Bamboo #5); target is a stretch — judge progress on the Beatable rivals we pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>king bamboo sheets</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>HOLD RANK</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #3, Pure Bamboo #8, KRIMANO #11, SONORO KATE (deep) #19, BC Bella Coterie #21</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>0.387</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — stretch target</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Only Aspirational rivals hold rank 10 or better (Bedsure (cooling) #3, Pure Bamboo #8); target is a stretch — judge progress on the Beatable rivals we pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>bamboo sheets full</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Hotel Sheets Direct #12, Bedsure (cooling) #13, Bedsure (organic) #16, KRIMANO #27, SONORO KATE (16in) #38</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>0.501</v>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — we lead the tracked field</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>We rank #11 organically, ahead of every tracked rival (best: Hotel Sheets Direct #12); the push is about the top rows untracked sellers hold. Target #2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>queen bamboo sheet set</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #4, Bambaw #10, KRIMANO #11, SONORO KATE (16in) #13, BAMPURE #17</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — stretch target</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>Only Aspirational rivals hold rank 6 or better (Bedsure (cooling) #4); target is a stretch — judge progress on the Beatable rivals we pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>bamboo king sheets</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>WAIT</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #4, KRIMANO #6, Pure Bamboo #9, Hotel Sheets Direct #18, SONORO KATE (deep) #27</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>0.413</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — reachable</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>KRIMANO #6 (Beatable) already holds a rank at or above target #9: the target is reachable for a listing like ours. Rivals to pass first: Hotel Sheets Direct #18.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>bamboo sheets queen</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #2, Bambaw #12, Pure Bamboo #13, KRIMANO #18, SONORO KATE (16in) #22</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>0.428</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — stretch target</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>Only Aspirational rivals hold rank 5 or better (Bedsure (cooling) #2); target is a stretch — judge progress on the Beatable rivals we pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>king sheets bamboo</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>KRIMANO #7, Pure Bamboo #10, SONORO KATE (deep) #15, Hotel Sheets Direct #22, SONORO KATE (16in) #28</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>0.406</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — reachable</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>KRIMANO #7 (Beatable) already holds a rank at or above target #10: the target is reachable for a listing like ours. Rivals to pass first: SONORO KATE (deep) #15, Hotel Sheets Direct #22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>viscose bamboo sheets</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>SONORO KATE (16in) #1, Pure Bamboo #5, KRIMANO #9, Bedsure (cooling) #11, Bambaw #14</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>0.257</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — reachable</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>SONORO KATE (16in) #1 (Beatable) already holds a rank at or above target #1: the target is reachable for a listing like ours. Rivals to pass first: Pure Bamboo #5, KRIMANO #9, Bedsure (cooling) #11, Bambaw #14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>king bed bamboo sheets</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Pure Bamboo #6, SONORO KATE (deep) #21, Hotel Sheets Direct #24, BC Bella Coterie #31, Bambaw #38</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>0.366</v>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — stretch target</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>Only Aspirational rivals hold rank 10 or better (Pure Bamboo #6); target is a stretch — judge progress on the Beatable rivals we pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>full size bamboo sheets</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>KRIMANO #11, Pure Bamboo #13, Bedsure (cooling) #15, Hotel Sheets Direct #24, BAMPURE #31</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>0.548</v>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>AGREES</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>The ranks between us (#29) and target (#10) are held by Beatable rivals (KRIMANO #11) — winnable ground.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>king bed sheets bamboo</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Pure Bamboo #5, KRIMANO #6, Hotel Sheets Direct #18, SONORO KATE (deep) #19, SONORO KATE (16in) #30</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>0.217</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — reachable</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>KRIMANO #6 (Beatable) already holds a rank at or above target #10: the target is reachable for a listing like ours. Rivals to pass first: Hotel Sheets Direct #18, SONORO KATE (deep) #19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>bamboo sheets with corner straps</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Bambaw #4, KRIMANO #7, BC Bella Coterie #15, GOKOTTA #17, Pure Bamboo #18</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>0.346</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>0.447</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AGREES</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>The ranks between us (#12) and target (#1) are held by Beatable rivals (Bambaw #4, KRIMANO #7) — winnable ground.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>bamboo full size bed sheets</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>PUSH</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling) #5, Pure Bamboo #8, KRIMANO #12, Hotel Sheets Direct #21, Bambaw #32</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>0.579</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>0.577</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AGREES — stretch target</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>Only Aspirational rivals hold rank 5 or better (Bedsure (cooling) #5); target is a stretch — judge progress on the Beatable rivals we pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Rivals</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Rival</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Call vs us</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Price from $</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Price to $</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Best listing units/30d</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>7-day traffic</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Traffic change</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>Paid share</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>SB keywords</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>Video keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Pure Bamboo</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Aspirational</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>not_beaten</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>109.99</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>109.99</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>21762</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>32557</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>2565055</v>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>-0.117</v>
+      </c>
+      <c r="K27" s="10" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L27" s="8" t="n">
+        <v>3791</v>
+      </c>
+      <c r="M27" s="8" t="n">
+        <v>2524</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Bedsure (cooling)</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Aspirational</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>not_beaten</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>69.69</v>
+      </c>
+      <c r="F28" s="8" t="n">
+        <v>64954</v>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H28" s="8" t="n">
+        <v>34342</v>
+      </c>
+      <c r="I28" s="8" t="n">
+        <v>2166046</v>
+      </c>
+      <c r="J28" s="10" t="n">
+        <v>-0.065</v>
+      </c>
+      <c r="K28" s="10" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="L28" s="8" t="n">
+        <v>2921</v>
+      </c>
+      <c r="M28" s="8" t="n">
+        <v>1646</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>BC Bella Coterie</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Beatable</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>not_beaten</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>134.99</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>134.99</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>5913</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>11726</v>
+      </c>
+      <c r="I29" s="8" t="n">
+        <v>591713</v>
+      </c>
+      <c r="J29" s="10" t="n">
+        <v>-0.152</v>
+      </c>
+      <c r="K29" s="10" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="L29" s="8" t="n">
+        <v>1390</v>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Hotel Sheets Direct</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Aspirational</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>not_beaten</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>79.98999999999999</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>94.98999999999999</v>
+      </c>
+      <c r="F30" s="8" t="n">
+        <v>37157</v>
+      </c>
+      <c r="G30" s="8" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H30" s="8" t="n">
+        <v>6616</v>
+      </c>
+      <c r="I30" s="8" t="n">
+        <v>451969</v>
+      </c>
+      <c r="J30" s="10" t="n">
+        <v>-0.109</v>
+      </c>
+      <c r="K30" s="10" t="n">
+        <v>0.393</v>
+      </c>
+      <c r="L30" s="8" t="n">
+        <v>933</v>
+      </c>
+      <c r="M30" s="8" t="n">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Bedsure (organic)</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Beatable</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>not_beaten</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>89.98999999999999</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>89.98999999999999</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>289</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="n">
+        <v>840292</v>
+      </c>
+      <c r="J31" s="10" t="n">
+        <v>-0.107</v>
+      </c>
+      <c r="K31" s="10" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="L31" s="8" t="n">
+        <v>2492</v>
+      </c>
+      <c r="M31" s="8" t="n">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>KRIMANO</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Beatable</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>not_beaten</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>68.39</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="G32" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H32" s="8" t="n">
+        <v>7202</v>
+      </c>
+      <c r="I32" s="8" t="n">
+        <v>390744</v>
+      </c>
+      <c r="J32" s="10" t="n">
+        <v>1.228</v>
+      </c>
+      <c r="K32" s="10" t="n">
+        <v>0.423</v>
+      </c>
+      <c r="L32" s="8" t="n">
+        <v>187</v>
+      </c>
+      <c r="M32" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>DOZ by SIJO</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Beatable</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>not_beaten</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>919</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>6681</v>
+      </c>
+      <c r="I33" s="8" t="n">
+        <v>171534</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <v>-0.073</v>
+      </c>
+      <c r="K33" s="10" t="n">
+        <v>0.446</v>
+      </c>
+      <c r="L33" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="M33" s="8" t="n">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Bambaw</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Beatable</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>not_beaten</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>2694</v>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H34" s="8" t="n">
+        <v>7968</v>
+      </c>
+      <c r="I34" s="8" t="n">
+        <v>407949</v>
+      </c>
+      <c r="J34" s="10" t="n">
+        <v>-0.185</v>
+      </c>
+      <c r="K34" s="10" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="L34" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M34" s="8" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>BAMPURE</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Beatable</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>beaten</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="F35" s="8" t="n">
+        <v>9032</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>1243</v>
+      </c>
+      <c r="I35" s="8" t="n">
+        <v>67699</v>
+      </c>
+      <c r="J35" s="10" t="n">
+        <v>-0.089</v>
+      </c>
+      <c r="K35" s="10" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="L35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>GOKOTTA</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Beatable</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>beaten</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>107</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>107</v>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>3233</v>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H36" s="8" t="n"/>
+      <c r="I36" s="8" t="n">
+        <v>76017</v>
+      </c>
+      <c r="J36" s="10" t="n">
+        <v>-0.237</v>
+      </c>
+      <c r="K36" s="10" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="L36" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="M36" s="8" t="n">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>SONORO KATE (deep)</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Beatable</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>not_beaten</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>3765</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>4455</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <v>185157</v>
+      </c>
+      <c r="J37" s="10" t="n">
+        <v>-0.149</v>
+      </c>
+      <c r="K37" s="10" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="L37" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Kickoff Home</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>beaten</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>76.98999999999999</v>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>76.98999999999999</v>
+      </c>
+      <c r="F38" s="8" t="n">
+        <v>681</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H38" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="I38" s="8" t="n">
+        <v>58169</v>
+      </c>
+      <c r="J38" s="8" t="n"/>
+      <c r="K38" s="10" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="L38" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="8" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>SONORO KATE (16in)</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Beatable</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F39" s="8" t="n">
+        <v>3904</v>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H39" s="8" t="n">
+        <v>1606</v>
+      </c>
+      <c r="I39" s="8" t="n">
+        <v>114504</v>
+      </c>
+      <c r="J39" s="10" t="n">
+        <v>-0.196</v>
+      </c>
+      <c r="K39" s="10" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="L39" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Full analysis — profiles, hero ASINs, all 2,266 market keywords, gaps, ASIN targets and the competitor rules — is in the decision engine reference workbook.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A41:J41"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -70357,791 +73313,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Negative keywords — one campaign per search term</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Every ranking term is bought by one exact campaign; broad, auto and phrase campaigns exclude it</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Seq</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Campaign</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Negatives now</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>After</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Terms added (negative exact)</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Our verdict</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="n">
-        <v>1738</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo sheets king size-[Bamboo|King]-(HSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>1 term(s)</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="n">
-        <v>1966</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo sheets king size-[Bamboo|King]-(HSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>36 term(s)</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>10 term(s)</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="n">
-        <v>1967</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo cooling sheets-[Bamboo|Cooling]-(MSV)-Broad-(DISC)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>13 term(s)</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>8 term(s)</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="n">
-        <v>1968</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo sheets queen size-[Bamboo|Queen]-(HSV)-Broad-(DISC)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>33 term(s)</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>7 term(s)</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="n">
-        <v>1969</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo sheets full-[Bamboo|Full]-(MSV)-Broad-(DISC)-DO-BAMBOO-FULL-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>20 term(s)</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>10 term(s)</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="n">
-        <v>1970</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>SP-Luxury Womens Gifts-(NOSV)-Broad-(Discovery)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>3 term(s)</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>3 term(s)</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="n">
-        <v>1971</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo sheets california king-[Bamboo|California King]-(LSV)-Broad-(DISC)-DO-BAMBOO-CALIFKING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>7 term(s)</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>4 term(s)</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="n">
-        <v>1972</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo sheets-[Bamboo]-(VHSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>0 term(s)</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>43 term(s)</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="n">
-        <v>1974</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>SP-Auto-(AUTO)-Auto-(Discovery)-DO-BAMBOO-KING-TAUPE-6PCS</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>127 term(s)</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>17 term(s)</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="n">
-        <v>1976</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>SP-Queen Sheets-(VHSV)-Broad-(Discovery)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>0 term(s)</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>15 term(s)</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="n">
-        <v>1977</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>SP-Auto-(AUTO)-Auto-(Discovery)-DO-BAMBOO-QUEEN-OLIVE-6PCS-3</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>18 term(s)</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>50 term(s)</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr"/>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="n">
-        <v>2142</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>SP-Decolure-(VLSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>10 term(s)</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>2 term(s)</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr"/>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Hold</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>brand negatives wait until the three brand exact campaigns are defensive and serving</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="n">
-        <v>2143</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo sheets california king-[Bamboo|California King]-(LSV)-Broad-(DISC)-DO-BAMBOO-CALIFKING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>7 term(s)</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>1 term(s)</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="n">
-        <v>2144</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>SP-Auto-(AUTO)-Auto-(Discovery)-DO-BAMBOO-KING-TAUPE-6PCS</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>127 term(s)</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>2 term(s)</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr"/>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="n">
-        <v>2145</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo sheets full-[Bamboo|Full]-(MSV)-Broad-(DISC)-DO-BAMBOO-FULL-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>20 term(s)</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>2 term(s)</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="n">
-        <v>2146</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo sheets-[Bamboo]-(VHSV)-Broad-(DISC)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>0 term(s)</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>1 term(s)</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr"/>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="n">
-        <v>2147</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>SP-bamboo cooling sheets-[Bamboo|Cooling]-(MSV)-Broad-(DISC)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>13 term(s)</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>1 term(s)</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr"/>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="n">
-        <v>2148</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>SP-Auto-(AUTO)-Auto-(Discovery)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>136 term(s)</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>1 term(s)</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Load</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>one campaign per term: excludes terms an exact campaign owns</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Also exclude “bamboo sheets” (negative exact) from every broad discovery campaign that still buys it; the “bamboo sheets” exact campaign owns it.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A24:J24"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="150" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Timeline — deal exit and the next events</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>When</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>What</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>29–30 Sep (deal)</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Load the 13 push terms (base + boost in one write, budgets by hand); cuts to break-even on non-push ranking campaigns; base cuts on conversions/discovery over break-even on 30 and 90 days; restart “bamboo sheets full”. Colour switches to White by hand on push campaigns first. Hold every new campaign, fold and the brand negatives.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>1 Oct — post-deal audit</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Confirm regular price; re-price on the full-price margin ($18.81). Re-evaluate the spend limit and the margin rule. Bring deal budgets down to each campaign’s required clicks at its new price. Decide the 17 builds, the restarts and the folds. Push carries on without a gap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>1–7 Oct — watch, don’t judge</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Deal-click sales keep arriving until ~7 Oct. Daily: spend vs limit, ad orders vs 14/day, top-of-search share on push campaigns, head-term ranks, Full White and Queen White stock. A head term falling &gt;10 places → find the cause before touching price.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>5 Oct</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>First weekly push tune.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>8–14 Oct — first clean read</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Re-run break-even on seven normal days. Mix check: where product pages still take &gt;20%, cut base again. Tune push on 12 Oct.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>15 Oct — Lightning Deal</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>One day. Don’t judge on it; keep push prices; check budgets won’t run out by mid-afternoon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>19 Oct</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Weekly tune. Goal: top 10 on at least half the push terms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>22–28 Oct — Best Deal</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Size the push for the deal a week ahead (price, clicks, budget, stock). The day-28 rank read skips deal days. Queen White arrival (1,002) lands 30 Oct.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>From early Nov</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Push into Prime / Black Friday–Cyber Monday: each event sized, funded and stock-checked at least three weeks ahead.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>